<commit_message>
Update attendance list ASS_CRN236396
Replace the Excel attendance sheet for ASS_CRN236396 with an updated binary version. This commit updates the spreadsheet content (Lista_Asistencia_ASS_CRN236396.xlsx) to reflect revised attendance data.
</commit_message>
<xml_diff>
--- a/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
+++ b/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ddf5fb2bc65e958/Documentos/GitHub/lc_arquitectura_de_sistemas_de_seguridad/Administracion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{702E06F4-7ABE-4278-9F4F-32BE2150E49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3CB0617-6449-4EB9-8BA4-E9A7FF29EB80}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{702E06F4-7ABE-4278-9F4F-32BE2150E49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F70B20E0-8ED9-4973-A91C-E751630F28CA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="149">
   <si>
     <t>LISTA DE ASISTENCIA — ARQUITECTURA DE SISTEMAS DE SEGURIDAD  |  Ciclo 2026-A  |  CRN 236396  |  Sección 401  |  Aula 101 Edif. 4L</t>
   </si>
@@ -847,6 +847,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1499,7 +1503,9 @@
       <c r="X6" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y6" s="12"/>
+      <c r="Y6" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z6" s="12"/>
       <c r="AA6" s="12"/>
       <c r="AB6" s="12"/>
@@ -1514,7 +1520,7 @@
       <c r="AK6" s="12"/>
       <c r="AL6" s="13">
         <f t="shared" ref="AL6:AL32" si="0">COUNTIF(F6,"A")+COUNTIF(G6,"A")+COUNTIF(H6,"A")+COUNTIF(I6,"A")+COUNTIF(J6,"A")+COUNTIF(K6,"A")+COUNTIF(L6,"A")+COUNTIF(M6,"A")+COUNTIF(N6,"A")+COUNTIF(O6,"A")+COUNTIF(P6,"A")+COUNTIF(Q6,"A")+COUNTIF(R6,"A")+COUNTIF(S6,"A")+COUNTIF(T6,"A")+COUNTIF(U6,"A")+COUNTIF(V6,"A")+COUNTIF(W6,"A")+COUNTIF(X6,"A")+COUNTIF(Y6,"A")+COUNTIF(Z6,"A")+COUNTIF(AA6,"A")+COUNTIF(AB6,"A")+COUNTIF(AC6,"A")+COUNTIF(AD6,"A")+COUNTIF(AE6,"A")+COUNTIF(AF6,"A")+COUNTIF(AG6,"A")+COUNTIF(AH6,"A")+COUNTIF(AI6,"A")+COUNTIF(AJ6,"A")+COUNTIF(AK6,"A")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM6" s="14">
         <f t="shared" ref="AM6:AM32" si="1">COUNTIF(F6,"F")+COUNTIF(G6,"F")+COUNTIF(H6,"F")+COUNTIF(I6,"F")+COUNTIF(J6,"F")+COUNTIF(K6,"F")+COUNTIF(L6,"F")+COUNTIF(M6,"F")+COUNTIF(N6,"F")+COUNTIF(O6,"F")+COUNTIF(P6,"F")+COUNTIF(Q6,"F")+COUNTIF(R6,"F")+COUNTIF(S6,"F")+COUNTIF(T6,"F")+COUNTIF(U6,"F")+COUNTIF(V6,"F")+COUNTIF(W6,"F")+COUNTIF(X6,"F")+COUNTIF(Y6,"F")+COUNTIF(Z6,"F")+COUNTIF(AA6,"F")+COUNTIF(AB6,"F")+COUNTIF(AC6,"F")+COUNTIF(AD6,"F")+COUNTIF(AE6,"F")+COUNTIF(AF6,"F")+COUNTIF(AG6,"F")+COUNTIF(AH6,"F")+COUNTIF(AI6,"F")+COUNTIF(AJ6,"F")+COUNTIF(AK6,"F")</f>
@@ -1522,7 +1528,7 @@
       </c>
       <c r="AN6" s="15">
         <f t="shared" ref="AN6:AN32" si="2">IF(AL6=0,"",AL6/32)</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="7" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1596,7 +1602,9 @@
       <c r="X7" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y7" s="19"/>
+      <c r="Y7" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z7" s="19"/>
       <c r="AA7" s="19"/>
       <c r="AB7" s="19"/>
@@ -1611,7 +1619,7 @@
       <c r="AK7" s="19"/>
       <c r="AL7" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM7" s="14">
         <f t="shared" si="1"/>
@@ -1619,7 +1627,7 @@
       </c>
       <c r="AN7" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="8" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1693,7 +1701,9 @@
       <c r="X8" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y8" s="12"/>
+      <c r="Y8" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z8" s="12"/>
       <c r="AA8" s="12"/>
       <c r="AB8" s="12"/>
@@ -1708,7 +1718,7 @@
       <c r="AK8" s="12"/>
       <c r="AL8" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM8" s="14">
         <f t="shared" si="1"/>
@@ -1716,7 +1726,7 @@
       </c>
       <c r="AN8" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="9" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1790,7 +1800,9 @@
       <c r="X9" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y9" s="19"/>
+      <c r="Y9" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z9" s="19"/>
       <c r="AA9" s="19"/>
       <c r="AB9" s="19"/>
@@ -1805,7 +1817,7 @@
       <c r="AK9" s="19"/>
       <c r="AL9" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM9" s="14">
         <f t="shared" si="1"/>
@@ -1813,7 +1825,7 @@
       </c>
       <c r="AN9" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="10" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1887,7 +1899,9 @@
       <c r="X10" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y10" s="12"/>
+      <c r="Y10" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z10" s="12"/>
       <c r="AA10" s="12"/>
       <c r="AB10" s="12"/>
@@ -1902,7 +1916,7 @@
       <c r="AK10" s="12"/>
       <c r="AL10" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM10" s="14">
         <f t="shared" si="1"/>
@@ -1910,7 +1924,7 @@
       </c>
       <c r="AN10" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="11" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1984,7 +1998,9 @@
       <c r="X11" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y11" s="19"/>
+      <c r="Y11" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z11" s="19"/>
       <c r="AA11" s="19"/>
       <c r="AB11" s="19"/>
@@ -1999,7 +2015,7 @@
       <c r="AK11" s="19"/>
       <c r="AL11" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM11" s="14">
         <f t="shared" si="1"/>
@@ -2007,7 +2023,7 @@
       </c>
       <c r="AN11" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="12" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2023,7 +2039,9 @@
       <c r="D12" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E12" s="11"/>
+      <c r="E12" s="11">
+        <v>1</v>
+      </c>
       <c r="F12" s="19" t="s">
         <v>145</v>
       </c>
@@ -2081,7 +2099,9 @@
       <c r="X12" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y12" s="12"/>
+      <c r="Y12" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z12" s="12"/>
       <c r="AA12" s="12"/>
       <c r="AB12" s="12"/>
@@ -2096,7 +2116,7 @@
       <c r="AK12" s="12"/>
       <c r="AL12" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM12" s="14">
         <f t="shared" si="1"/>
@@ -2104,7 +2124,7 @@
       </c>
       <c r="AN12" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="13" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2178,7 +2198,9 @@
       <c r="X13" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y13" s="19"/>
+      <c r="Y13" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z13" s="19"/>
       <c r="AA13" s="19"/>
       <c r="AB13" s="19"/>
@@ -2193,7 +2215,7 @@
       <c r="AK13" s="19"/>
       <c r="AL13" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM13" s="14">
         <f t="shared" si="1"/>
@@ -2201,7 +2223,7 @@
       </c>
       <c r="AN13" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="14" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2275,7 +2297,9 @@
       <c r="X14" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y14" s="12"/>
+      <c r="Y14" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z14" s="12"/>
       <c r="AA14" s="12"/>
       <c r="AB14" s="12"/>
@@ -2290,7 +2314,7 @@
       <c r="AK14" s="12"/>
       <c r="AL14" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM14" s="14">
         <f t="shared" si="1"/>
@@ -2298,7 +2322,7 @@
       </c>
       <c r="AN14" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="15" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2314,7 +2338,9 @@
       <c r="D15" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="18">
+        <v>1</v>
+      </c>
       <c r="F15" s="19" t="s">
         <v>145</v>
       </c>
@@ -2372,7 +2398,9 @@
       <c r="X15" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y15" s="19"/>
+      <c r="Y15" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z15" s="19"/>
       <c r="AA15" s="19"/>
       <c r="AB15" s="19"/>
@@ -2387,7 +2415,7 @@
       <c r="AK15" s="19"/>
       <c r="AL15" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM15" s="14">
         <f t="shared" si="1"/>
@@ -2395,7 +2423,7 @@
       </c>
       <c r="AN15" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="16" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2469,7 +2497,9 @@
       <c r="X16" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y16" s="12"/>
+      <c r="Y16" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z16" s="12"/>
       <c r="AA16" s="12"/>
       <c r="AB16" s="12"/>
@@ -2484,7 +2514,7 @@
       <c r="AK16" s="12"/>
       <c r="AL16" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM16" s="14">
         <f t="shared" si="1"/>
@@ -2492,7 +2522,7 @@
       </c>
       <c r="AN16" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="17" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2566,7 +2596,9 @@
       <c r="X17" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y17" s="19"/>
+      <c r="Y17" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z17" s="19"/>
       <c r="AA17" s="19"/>
       <c r="AB17" s="19"/>
@@ -2581,7 +2613,7 @@
       <c r="AK17" s="19"/>
       <c r="AL17" s="13">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AM17" s="14">
         <f t="shared" si="1"/>
@@ -2589,7 +2621,7 @@
       </c>
       <c r="AN17" s="15">
         <f t="shared" si="2"/>
-        <v>0.53125</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="18" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2663,7 +2695,9 @@
       <c r="X18" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y18" s="12"/>
+      <c r="Y18" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z18" s="12"/>
       <c r="AA18" s="12"/>
       <c r="AB18" s="12"/>
@@ -2678,7 +2712,7 @@
       <c r="AK18" s="12"/>
       <c r="AL18" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM18" s="14">
         <f t="shared" si="1"/>
@@ -2686,7 +2720,7 @@
       </c>
       <c r="AN18" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="19" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2702,7 +2736,9 @@
       <c r="D19" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="18">
+        <v>1</v>
+      </c>
       <c r="F19" s="19" t="s">
         <v>145</v>
       </c>
@@ -2760,7 +2796,9 @@
       <c r="X19" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y19" s="19"/>
+      <c r="Y19" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z19" s="19"/>
       <c r="AA19" s="19"/>
       <c r="AB19" s="19"/>
@@ -2775,7 +2813,7 @@
       <c r="AK19" s="19"/>
       <c r="AL19" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM19" s="14">
         <f t="shared" si="1"/>
@@ -2783,7 +2821,7 @@
       </c>
       <c r="AN19" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="20" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2857,7 +2895,9 @@
       <c r="X20" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y20" s="12"/>
+      <c r="Y20" s="12" t="s">
+        <v>147</v>
+      </c>
       <c r="Z20" s="12"/>
       <c r="AA20" s="12"/>
       <c r="AB20" s="12"/>
@@ -2876,7 +2916,7 @@
       </c>
       <c r="AM20" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN20" s="15">
         <f t="shared" si="2"/>
@@ -2954,7 +2994,9 @@
       <c r="X21" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y21" s="19"/>
+      <c r="Y21" s="19" t="s">
+        <v>147</v>
+      </c>
       <c r="Z21" s="19"/>
       <c r="AA21" s="19"/>
       <c r="AB21" s="19"/>
@@ -2973,7 +3015,7 @@
       </c>
       <c r="AM21" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN21" s="15">
         <f t="shared" si="2"/>
@@ -3051,7 +3093,9 @@
       <c r="X22" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y22" s="12"/>
+      <c r="Y22" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z22" s="12"/>
       <c r="AA22" s="12"/>
       <c r="AB22" s="12"/>
@@ -3066,7 +3110,7 @@
       <c r="AK22" s="12"/>
       <c r="AL22" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM22" s="14">
         <f t="shared" si="1"/>
@@ -3074,7 +3118,7 @@
       </c>
       <c r="AN22" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="23" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3148,7 +3192,9 @@
       <c r="X23" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y23" s="19"/>
+      <c r="Y23" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z23" s="19"/>
       <c r="AA23" s="19"/>
       <c r="AB23" s="19"/>
@@ -3163,7 +3209,7 @@
       <c r="AK23" s="19"/>
       <c r="AL23" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM23" s="14">
         <f t="shared" si="1"/>
@@ -3171,7 +3217,7 @@
       </c>
       <c r="AN23" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="24" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3245,7 +3291,9 @@
       <c r="X24" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y24" s="12"/>
+      <c r="Y24" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z24" s="12"/>
       <c r="AA24" s="12"/>
       <c r="AB24" s="12"/>
@@ -3260,7 +3308,7 @@
       <c r="AK24" s="12"/>
       <c r="AL24" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM24" s="14">
         <f t="shared" si="1"/>
@@ -3268,7 +3316,7 @@
       </c>
       <c r="AN24" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="25" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3342,7 +3390,9 @@
       <c r="X25" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y25" s="19"/>
+      <c r="Y25" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z25" s="19"/>
       <c r="AA25" s="19"/>
       <c r="AB25" s="19"/>
@@ -3357,7 +3407,7 @@
       <c r="AK25" s="19"/>
       <c r="AL25" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM25" s="14">
         <f t="shared" si="1"/>
@@ -3365,7 +3415,7 @@
       </c>
       <c r="AN25" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="26" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3439,7 +3489,9 @@
       <c r="X26" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y26" s="12"/>
+      <c r="Y26" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z26" s="12"/>
       <c r="AA26" s="12"/>
       <c r="AB26" s="12"/>
@@ -3454,7 +3506,7 @@
       <c r="AK26" s="12"/>
       <c r="AL26" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM26" s="14">
         <f t="shared" si="1"/>
@@ -3462,7 +3514,7 @@
       </c>
       <c r="AN26" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="27" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3536,7 +3588,9 @@
       <c r="X27" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y27" s="19"/>
+      <c r="Y27" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z27" s="19"/>
       <c r="AA27" s="19"/>
       <c r="AB27" s="19"/>
@@ -3551,7 +3605,7 @@
       <c r="AK27" s="19"/>
       <c r="AL27" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM27" s="14">
         <f t="shared" si="1"/>
@@ -3559,7 +3613,7 @@
       </c>
       <c r="AN27" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="28" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3633,7 +3687,9 @@
       <c r="X28" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y28" s="12"/>
+      <c r="Y28" s="12" t="s">
+        <v>147</v>
+      </c>
       <c r="Z28" s="12"/>
       <c r="AA28" s="12"/>
       <c r="AB28" s="12"/>
@@ -3652,7 +3708,7 @@
       </c>
       <c r="AM28" s="14">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN28" s="15">
         <f t="shared" si="2"/>
@@ -3730,7 +3786,9 @@
       <c r="X29" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y29" s="19"/>
+      <c r="Y29" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z29" s="19"/>
       <c r="AA29" s="19"/>
       <c r="AB29" s="19"/>
@@ -3745,7 +3803,7 @@
       <c r="AK29" s="19"/>
       <c r="AL29" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM29" s="14">
         <f t="shared" si="1"/>
@@ -3753,7 +3811,7 @@
       </c>
       <c r="AN29" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="30" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3769,7 +3827,9 @@
       <c r="D30" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="11"/>
+      <c r="E30" s="11">
+        <v>1</v>
+      </c>
       <c r="F30" s="19" t="s">
         <v>145</v>
       </c>
@@ -3827,7 +3887,9 @@
       <c r="X30" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y30" s="12"/>
+      <c r="Y30" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z30" s="12"/>
       <c r="AA30" s="12"/>
       <c r="AB30" s="12"/>
@@ -3842,7 +3904,7 @@
       <c r="AK30" s="12"/>
       <c r="AL30" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM30" s="14">
         <f t="shared" si="1"/>
@@ -3850,7 +3912,7 @@
       </c>
       <c r="AN30" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="31" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3866,7 +3928,9 @@
       <c r="D31" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="E31" s="18"/>
+      <c r="E31" s="18">
+        <v>1</v>
+      </c>
       <c r="F31" s="19" t="s">
         <v>145</v>
       </c>
@@ -3924,7 +3988,9 @@
       <c r="X31" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y31" s="19"/>
+      <c r="Y31" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="Z31" s="19"/>
       <c r="AA31" s="19"/>
       <c r="AB31" s="19"/>
@@ -3939,7 +4005,7 @@
       <c r="AK31" s="19"/>
       <c r="AL31" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM31" s="14">
         <f t="shared" si="1"/>
@@ -3947,7 +4013,7 @@
       </c>
       <c r="AN31" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="32" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3963,7 +4029,9 @@
       <c r="D32" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="E32" s="11"/>
+      <c r="E32" s="11">
+        <v>1</v>
+      </c>
       <c r="F32" s="19" t="s">
         <v>145</v>
       </c>
@@ -4021,7 +4089,9 @@
       <c r="X32" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y32" s="12"/>
+      <c r="Y32" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="Z32" s="12"/>
       <c r="AA32" s="12"/>
       <c r="AB32" s="12"/>
@@ -4036,7 +4106,7 @@
       <c r="AK32" s="12"/>
       <c r="AL32" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AM32" s="14">
         <f t="shared" si="1"/>
@@ -4044,7 +4114,7 @@
       </c>
       <c r="AN32" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
     </row>
     <row r="33" spans="1:40" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4133,7 +4203,7 @@
       </c>
       <c r="Y33" s="20">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Z33" s="20">
         <f t="shared" si="3"/>
@@ -4233,11 +4303,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="AH3:AI3"/>
     <mergeCell ref="AJ3:AK3"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A34:AN34"/>
@@ -4253,6 +4318,11 @@
     <mergeCell ref="T3:U3"/>
     <mergeCell ref="V3:W3"/>
     <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="AB3:AC3"/>
+    <mergeCell ref="AD3:AE3"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="AH3:AI3"/>
   </mergeCells>
   <conditionalFormatting sqref="AN6:AN32">
     <cfRule type="expression" dxfId="1" priority="2">
@@ -4334,7 +4404,7 @@
       </c>
       <c r="E3" s="13">
         <f>Asistencia!AL6</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="14">
         <f>Asistencia!AM6</f>
@@ -4342,7 +4412,7 @@
       </c>
       <c r="G3" s="15">
         <f>Asistencia!AN6</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H3" s="9" t="str">
         <f>IF(Asistencia!AN6="","Sin datos",IF(Asistencia!AN6&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4364,7 +4434,7 @@
       </c>
       <c r="E4" s="13">
         <f>Asistencia!AL7</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" s="14">
         <f>Asistencia!AM7</f>
@@ -4372,7 +4442,7 @@
       </c>
       <c r="G4" s="15">
         <f>Asistencia!AN7</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H4" s="16" t="str">
         <f>IF(Asistencia!AN7="","Sin datos",IF(Asistencia!AN7&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4394,7 +4464,7 @@
       </c>
       <c r="E5" s="13">
         <f>Asistencia!AL8</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F5" s="14">
         <f>Asistencia!AM8</f>
@@ -4402,7 +4472,7 @@
       </c>
       <c r="G5" s="15">
         <f>Asistencia!AN8</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H5" s="9" t="str">
         <f>IF(Asistencia!AN8="","Sin datos",IF(Asistencia!AN8&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4424,7 +4494,7 @@
       </c>
       <c r="E6" s="13">
         <f>Asistencia!AL9</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F6" s="14">
         <f>Asistencia!AM9</f>
@@ -4432,7 +4502,7 @@
       </c>
       <c r="G6" s="15">
         <f>Asistencia!AN9</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H6" s="16" t="str">
         <f>IF(Asistencia!AN9="","Sin datos",IF(Asistencia!AN9&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4454,7 +4524,7 @@
       </c>
       <c r="E7" s="13">
         <f>Asistencia!AL10</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" s="14">
         <f>Asistencia!AM10</f>
@@ -4462,7 +4532,7 @@
       </c>
       <c r="G7" s="15">
         <f>Asistencia!AN10</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H7" s="9" t="str">
         <f>IF(Asistencia!AN10="","Sin datos",IF(Asistencia!AN10&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4484,7 +4554,7 @@
       </c>
       <c r="E8" s="13">
         <f>Asistencia!AL11</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F8" s="14">
         <f>Asistencia!AM11</f>
@@ -4492,7 +4562,7 @@
       </c>
       <c r="G8" s="15">
         <f>Asistencia!AN11</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H8" s="16" t="str">
         <f>IF(Asistencia!AN11="","Sin datos",IF(Asistencia!AN11&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4514,7 +4584,7 @@
       </c>
       <c r="E9" s="13">
         <f>Asistencia!AL12</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F9" s="14">
         <f>Asistencia!AM12</f>
@@ -4522,7 +4592,7 @@
       </c>
       <c r="G9" s="15">
         <f>Asistencia!AN12</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H9" s="9" t="str">
         <f>IF(Asistencia!AN12="","Sin datos",IF(Asistencia!AN12&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4544,7 +4614,7 @@
       </c>
       <c r="E10" s="13">
         <f>Asistencia!AL13</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F10" s="14">
         <f>Asistencia!AM13</f>
@@ -4552,7 +4622,7 @@
       </c>
       <c r="G10" s="15">
         <f>Asistencia!AN13</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H10" s="16" t="str">
         <f>IF(Asistencia!AN13="","Sin datos",IF(Asistencia!AN13&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4574,7 +4644,7 @@
       </c>
       <c r="E11" s="13">
         <f>Asistencia!AL14</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F11" s="14">
         <f>Asistencia!AM14</f>
@@ -4582,7 +4652,7 @@
       </c>
       <c r="G11" s="15">
         <f>Asistencia!AN14</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H11" s="9" t="str">
         <f>IF(Asistencia!AN14="","Sin datos",IF(Asistencia!AN14&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4604,7 +4674,7 @@
       </c>
       <c r="E12" s="13">
         <f>Asistencia!AL15</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F12" s="14">
         <f>Asistencia!AM15</f>
@@ -4612,7 +4682,7 @@
       </c>
       <c r="G12" s="15">
         <f>Asistencia!AN15</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H12" s="16" t="str">
         <f>IF(Asistencia!AN15="","Sin datos",IF(Asistencia!AN15&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4634,7 +4704,7 @@
       </c>
       <c r="E13" s="13">
         <f>Asistencia!AL16</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F13" s="14">
         <f>Asistencia!AM16</f>
@@ -4642,7 +4712,7 @@
       </c>
       <c r="G13" s="15">
         <f>Asistencia!AN16</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H13" s="9" t="str">
         <f>IF(Asistencia!AN16="","Sin datos",IF(Asistencia!AN16&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4664,7 +4734,7 @@
       </c>
       <c r="E14" s="13">
         <f>Asistencia!AL17</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F14" s="14">
         <f>Asistencia!AM17</f>
@@ -4672,7 +4742,7 @@
       </c>
       <c r="G14" s="15">
         <f>Asistencia!AN17</f>
-        <v>0.53125</v>
+        <v>0.5625</v>
       </c>
       <c r="H14" s="16" t="str">
         <f>IF(Asistencia!AN17="","Sin datos",IF(Asistencia!AN17&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4694,7 +4764,7 @@
       </c>
       <c r="E15" s="13">
         <f>Asistencia!AL18</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F15" s="14">
         <f>Asistencia!AM18</f>
@@ -4702,7 +4772,7 @@
       </c>
       <c r="G15" s="15">
         <f>Asistencia!AN18</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H15" s="9" t="str">
         <f>IF(Asistencia!AN18="","Sin datos",IF(Asistencia!AN18&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4724,7 +4794,7 @@
       </c>
       <c r="E16" s="13">
         <f>Asistencia!AL19</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F16" s="14">
         <f>Asistencia!AM19</f>
@@ -4732,7 +4802,7 @@
       </c>
       <c r="G16" s="15">
         <f>Asistencia!AN19</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H16" s="16" t="str">
         <f>IF(Asistencia!AN19="","Sin datos",IF(Asistencia!AN19&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4758,7 +4828,7 @@
       </c>
       <c r="F17" s="14">
         <f>Asistencia!AM20</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="15">
         <f>Asistencia!AN20</f>
@@ -4788,7 +4858,7 @@
       </c>
       <c r="F18" s="14">
         <f>Asistencia!AM21</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="15">
         <f>Asistencia!AN21</f>
@@ -4814,7 +4884,7 @@
       </c>
       <c r="E19" s="13">
         <f>Asistencia!AL22</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F19" s="14">
         <f>Asistencia!AM22</f>
@@ -4822,7 +4892,7 @@
       </c>
       <c r="G19" s="15">
         <f>Asistencia!AN22</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H19" s="9" t="str">
         <f>IF(Asistencia!AN22="","Sin datos",IF(Asistencia!AN22&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4844,7 +4914,7 @@
       </c>
       <c r="E20" s="13">
         <f>Asistencia!AL23</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F20" s="14">
         <f>Asistencia!AM23</f>
@@ -4852,7 +4922,7 @@
       </c>
       <c r="G20" s="15">
         <f>Asistencia!AN23</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H20" s="16" t="str">
         <f>IF(Asistencia!AN23="","Sin datos",IF(Asistencia!AN23&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4874,7 +4944,7 @@
       </c>
       <c r="E21" s="13">
         <f>Asistencia!AL24</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F21" s="14">
         <f>Asistencia!AM24</f>
@@ -4882,7 +4952,7 @@
       </c>
       <c r="G21" s="15">
         <f>Asistencia!AN24</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H21" s="9" t="str">
         <f>IF(Asistencia!AN24="","Sin datos",IF(Asistencia!AN24&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4904,7 +4974,7 @@
       </c>
       <c r="E22" s="13">
         <f>Asistencia!AL25</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F22" s="14">
         <f>Asistencia!AM25</f>
@@ -4912,7 +4982,7 @@
       </c>
       <c r="G22" s="15">
         <f>Asistencia!AN25</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H22" s="16" t="str">
         <f>IF(Asistencia!AN25="","Sin datos",IF(Asistencia!AN25&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4934,7 +5004,7 @@
       </c>
       <c r="E23" s="13">
         <f>Asistencia!AL26</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F23" s="14">
         <f>Asistencia!AM26</f>
@@ -4942,7 +5012,7 @@
       </c>
       <c r="G23" s="15">
         <f>Asistencia!AN26</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H23" s="9" t="str">
         <f>IF(Asistencia!AN26="","Sin datos",IF(Asistencia!AN26&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4964,7 +5034,7 @@
       </c>
       <c r="E24" s="13">
         <f>Asistencia!AL27</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F24" s="14">
         <f>Asistencia!AM27</f>
@@ -4972,7 +5042,7 @@
       </c>
       <c r="G24" s="15">
         <f>Asistencia!AN27</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H24" s="16" t="str">
         <f>IF(Asistencia!AN27="","Sin datos",IF(Asistencia!AN27&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4998,7 +5068,7 @@
       </c>
       <c r="F25" s="14">
         <f>Asistencia!AM28</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15">
         <f>Asistencia!AN28</f>
@@ -5024,7 +5094,7 @@
       </c>
       <c r="E26" s="13">
         <f>Asistencia!AL29</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F26" s="14">
         <f>Asistencia!AM29</f>
@@ -5032,7 +5102,7 @@
       </c>
       <c r="G26" s="15">
         <f>Asistencia!AN29</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H26" s="16" t="str">
         <f>IF(Asistencia!AN29="","Sin datos",IF(Asistencia!AN29&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5054,7 +5124,7 @@
       </c>
       <c r="E27" s="13">
         <f>Asistencia!AL30</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F27" s="14">
         <f>Asistencia!AM30</f>
@@ -5062,7 +5132,7 @@
       </c>
       <c r="G27" s="15">
         <f>Asistencia!AN30</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H27" s="9" t="str">
         <f>IF(Asistencia!AN30="","Sin datos",IF(Asistencia!AN30&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5084,7 +5154,7 @@
       </c>
       <c r="E28" s="13">
         <f>Asistencia!AL31</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F28" s="14">
         <f>Asistencia!AM31</f>
@@ -5092,7 +5162,7 @@
       </c>
       <c r="G28" s="15">
         <f>Asistencia!AN31</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H28" s="16" t="str">
         <f>IF(Asistencia!AN31="","Sin datos",IF(Asistencia!AN31&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5114,7 +5184,7 @@
       </c>
       <c r="E29" s="13">
         <f>Asistencia!AL32</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F29" s="14">
         <f>Asistencia!AM32</f>
@@ -5122,7 +5192,7 @@
       </c>
       <c r="G29" s="15">
         <f>Asistencia!AN32</f>
-        <v>0.5625</v>
+        <v>0.59375</v>
       </c>
       <c r="H29" s="9" t="str">
         <f>IF(Asistencia!AN32="","Sin datos",IF(Asistencia!AN32&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>

</xml_diff>